<commit_message>
Update Israel to latest Oct 2026 polls (Yashar! / Gadi Eisenkot) and replace Russia with Spain (350-seat Congreso + 18-region map)
</commit_message>
<xml_diff>
--- a/election_simulator_parties.xlsx
+++ b/election_simulator_parties.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Israel" sheetId="8" r:id="rId8"/>
     <sheet name="Canada" sheetId="9" r:id="rId9"/>
     <sheet name="Italy" sheetId="10" r:id="rId10"/>
-    <sheet name="Russia" sheetId="11" r:id="rId11"/>
+    <sheet name="Spain" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -1668,282 +1668,564 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="0">
         <is>
-          <t>kharitonov</t>
+          <t>PODEMOS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="0">
         <is>
-          <t>CPRF</t>
+          <t>Podemos</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="0">
         <is>
-          <t>Communist Party of the Russian Federation (CPRF)</t>
+          <t>Podemos</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="0">
         <is>
-          <t>Nikolay Kharitonov</t>
+          <t>Ione Belarra / Irene Montero</t>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="0">
         <is>
-          <t>2024 Presidential</t>
+          <t>2023–2026 Congreso</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="0">
         <is>
-          <t>Far-left (Socially conservative)</t>
+          <t>Left-wing to Far-left</t>
         </is>
       </c>
       <c r="G2" t="inlineStr" s="0">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="H2" t="inlineStr" s="0">
         <is>
-          <t>Communism, Marxism-Leninism, Soviet patriotism</t>
+          <t>Left-wing populism, Democratic socialism, Feminism</t>
         </is>
       </c>
       <c r="I2" t="inlineStr" s="0">
         <is>
-          <t>Systemic opposition</t>
+          <t>Left bloc</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr" s="0">
         <is>
-          <t>duntsova</t>
+          <t>BILDU</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="0">
         <is>
-          <t>Duntsova</t>
+          <t>EH Bildu</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="0">
         <is>
-          <t>Independent Democratic Opposition</t>
+          <t>Euskal Herria Bildu</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="0">
         <is>
-          <t>Yekaterina Duntsova</t>
+          <t>Arnaldo Otegi / Mertxe Aizpurua</t>
         </is>
       </c>
       <c r="E3" t="inlineStr" s="0">
         <is>
-          <t>2024 Presidential (Scenario)</t>
+          <t>2023–2026 Congreso</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="0">
         <is>
-          <t>Centre-left to Centre</t>
+          <t>Left-wing</t>
         </is>
       </c>
       <c r="G3" t="inlineStr" s="0">
         <is>
-          <t>4.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr" s="0">
         <is>
-          <t>Social liberalism, Peace platform, Decentralization</t>
+          <t>Basque nationalism, Basque independence, Democratic socialism</t>
         </is>
       </c>
       <c r="I3" t="inlineStr" s="0">
         <is>
-          <t>Non-systemic opposition</t>
+          <t>Regional Left</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr" s="0">
         <is>
-          <t>nadezhdin</t>
+          <t>ERC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr" s="0">
         <is>
-          <t>Civic Init.</t>
+          <t>ERC</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="0">
         <is>
-          <t>Civic Initiative (Grazhdanskaya Initsiativa)</t>
+          <t>Esquerra Republicana de Catalunya</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="0">
         <is>
-          <t>Boris Nadezhdin</t>
+          <t>Oriol Junqueras / Gabriel Rufián</t>
         </is>
       </c>
       <c r="E4" t="inlineStr" s="0">
         <is>
-          <t>2024 Presidential (Scenario)</t>
+          <t>2023–2026 Congreso</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="0">
         <is>
-          <t>Centre to Centre-right</t>
+          <t>Left-wing</t>
         </is>
       </c>
       <c r="G4" t="inlineStr" s="0">
         <is>
-          <t>5.2</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="H4" t="inlineStr" s="0">
         <is>
-          <t>Liberal democracy, Constitutionalism, Anti-war reformism</t>
+          <t>Catalan independence, Catalan republicanism, Social democracy</t>
         </is>
       </c>
       <c r="I4" t="inlineStr" s="0">
         <is>
-          <t>Non-systemic opposition</t>
+          <t>Regional Left</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr" s="0">
         <is>
-          <t>davankov</t>
+          <t>SUMAR</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="0">
         <is>
-          <t>New People</t>
+          <t>Sumar</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="0">
         <is>
-          <t>New People (Novye Lyudi)</t>
+          <t>Movimiento Sumar &amp; Allies</t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="0">
         <is>
-          <t>Vladislav Davankov</t>
+          <t>Yolanda Díaz</t>
         </is>
       </c>
       <c r="E5" t="inlineStr" s="0">
         <is>
-          <t>2024 Presidential</t>
+          <t>2023–2026 Congreso</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="0">
         <is>
-          <t>Centre-right</t>
+          <t>Left-wing</t>
         </is>
       </c>
       <c r="G5" t="inlineStr" s="0">
         <is>
-          <t>5.8</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr" s="0">
         <is>
-          <t>Liberalism, Entrepreneurship, Moderate modernization</t>
+          <t>Democratic socialism, Green politics, Progressivism, Labor rights</t>
         </is>
       </c>
       <c r="I5" t="inlineStr" s="0">
         <is>
-          <t>Systemic opposition</t>
+          <t>Left bloc</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="0">
         <is>
-          <t>putin</t>
+          <t>BNG</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="0">
         <is>
-          <t>Putin (ONF)</t>
+          <t>BNG</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="0">
         <is>
-          <t>Independent / United Russia (All-Russian People's Front)</t>
+          <t>Bloque Nacionalista Galego</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="0">
         <is>
-          <t>Vladimir Putin</t>
+          <t>Ana Pontón / Néstor Rego</t>
         </is>
       </c>
       <c r="E6" t="inlineStr" s="0">
         <is>
-          <t>2024 Presidential</t>
+          <t>2023–2026 Congreso</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="0">
         <is>
-          <t>Right-wing</t>
+          <t>Left-wing</t>
         </is>
       </c>
       <c r="G6" t="inlineStr" s="0">
         <is>
-          <t>7.8</t>
+          <t>2.6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr" s="0">
         <is>
-          <t>Russian nationalism, Statism, Conservatism, Sovereign democracy</t>
+          <t>Galician nationalism, Socialism, Euroscepticism</t>
         </is>
       </c>
       <c r="I6" t="inlineStr" s="0">
         <is>
-          <t>Incumbent</t>
+          <t>Regional Left</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr" s="0">
         <is>
-          <t>slutsky</t>
+          <t>PSOE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="0">
         <is>
-          <t>LDPR</t>
+          <t>PSOE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="0">
         <is>
-          <t>Liberal Democratic Party of Russia (LDPR)</t>
+          <t>Partido Socialista Obrero Español (PSOE)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="0">
         <is>
-          <t>Leonid Slutsky</t>
+          <t>Pedro Sánchez</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="0">
         <is>
-          <t>2024 Presidential</t>
+          <t>2023–2026 Congreso</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="0">
         <is>
+          <t>Centre-left</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr" s="0">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr" s="0">
+        <is>
+          <t>Social democracy, Pro-Europeanism, Federalism</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr" s="0">
+        <is>
+          <t>Left bloc</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="0">
+        <is>
+          <t>PNV</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="0">
+        <is>
+          <t>EAJ-PNV</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="0">
+        <is>
+          <t>Partido Nacionalista Vasco (EAJ-PNV)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="0">
+        <is>
+          <t>Aitor Esteban / Andoni Ortuzar</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="0">
+        <is>
+          <t>2023–2026 Congreso</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="0">
+        <is>
+          <t>Centre to Centre-right</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr" s="0">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr" s="0">
+        <is>
+          <t>Basque nationalism, Christian democracy, Liberalism</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr" s="0">
+        <is>
+          <t>Regional Centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="0">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="0">
+        <is>
+          <t>CC / Reg.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="0">
+        <is>
+          <t>Coalición Canaria &amp; Regionalists (UPN)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="0">
+        <is>
+          <t>Fernando Clavijo / Cristina Valido</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="0">
+        <is>
+          <t>2023–2026 Congreso</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="0">
+        <is>
+          <t>Centre to Centre-right</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr" s="0">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr" s="0">
+        <is>
+          <t>Canary regionalism, Centrism, Autonomy</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr" s="0">
+        <is>
+          <t>Regional Centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="0">
+        <is>
+          <t>JUNTS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="0">
+        <is>
+          <t>Junts</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="0">
+        <is>
+          <t>Junts per Catalunya</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="0">
+        <is>
+          <t>Carles Puigdemont / Míriam Nogueras</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="0">
+        <is>
+          <t>2023–2026 Congreso</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="0">
+        <is>
+          <t>Centre-right</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr" s="0">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr" s="0">
+        <is>
+          <t>Catalan independence, Liberal conservatism</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr" s="0">
+        <is>
+          <t>Regional Right</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="0">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="0">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="0">
+        <is>
+          <t>Partido Popular (People's Party)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="0">
+        <is>
+          <t>Alberto Núñez Feijóo</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="0">
+        <is>
+          <t>2023–2026 Congreso</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="0">
+        <is>
+          <t>Centre-right to Right-wing</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr" s="0">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr" s="0">
+        <is>
+          <t>Conservatism, Christian democracy, Economic liberalism, Spanish unionism</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr" s="0">
+        <is>
+          <t>Right bloc</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="0">
+        <is>
+          <t>VOX</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="0">
+        <is>
+          <t>Vox</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="0">
+        <is>
+          <t>Vox</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="0">
+        <is>
+          <t>Santiago Abascal</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="0">
+        <is>
+          <t>2023–2026 Congreso</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr" s="0">
+        <is>
+          <t>Right-wing to Far-right</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr" s="0">
+        <is>
+          <t>8.9</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr" s="0">
+        <is>
+          <t>Spanish ultranationalism, National conservatism, Right-wing populism</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr" s="0">
+        <is>
+          <t>Right bloc</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr" s="0">
+        <is>
+          <t>SALF</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="0">
+        <is>
+          <t>SALF</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="0">
+        <is>
+          <t>Se Acabó la Fiesta (SALF)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="0">
+        <is>
+          <t>Alvise Pérez</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="0">
+        <is>
+          <t>2026 Polls</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr" s="0">
+        <is>
           <t>Far-right</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr" s="0">
-        <is>
-          <t>9.0</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr" s="0">
-        <is>
-          <t>Russian ultranationalism, Imperialism, Right-wing populism</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr" s="0">
-        <is>
-          <t>Systemic opposition</t>
+      <c r="G13" t="inlineStr" s="0">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr" s="0">
+        <is>
+          <t>Anti-establishment populism, Anti-corruption, Right-wing populism</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr" s="0">
+        <is>
+          <t>Right bloc</t>
         </is>
       </c>
     </row>
@@ -5641,7 +5923,7 @@
       </c>
       <c r="I4" t="inlineStr" s="0">
         <is>
-          <t>Opposition / Swing</t>
+          <t>Arab / Swing</t>
         </is>
       </c>
     </row>
@@ -5742,22 +6024,22 @@
     <row r="7">
       <c r="A7" t="inlineStr" s="0">
         <is>
-          <t>NU</t>
+          <t>YASHAR</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="0">
         <is>
-          <t>National Unity</t>
+          <t>Yashar! (Eisenkot)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="0">
         <is>
-          <t>National Unity (Blue and White)</t>
+          <t>Yashar! with Eisenkot (Straight!)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="0">
         <is>
-          <t>Benny Gantz</t>
+          <t>Gadi Eisenkot</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="0">
@@ -5767,17 +6049,17 @@
       </c>
       <c r="F7" t="inlineStr" s="0">
         <is>
-          <t>Centre to Centre-right</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="G7" t="inlineStr" s="0">
         <is>
-          <t>5.5</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr" s="0">
         <is>
-          <t>Statism (Mamlachtiyut), Liberal conservatism, Pragmatism</t>
+          <t>Centrism, National security, Institutionalism, Liberal Zionism</t>
         </is>
       </c>
       <c r="I7" t="inlineStr" s="0">
@@ -5789,22 +6071,22 @@
     <row r="8">
       <c r="A8" t="inlineStr" s="0">
         <is>
-          <t>BENNETT</t>
+          <t>NU</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="0">
         <is>
-          <t>Bennett 2026</t>
+          <t>Blue &amp; White</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t>Bennett 2026 (New Right)</t>
+          <t>National Unity (Blue and White)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="0">
         <is>
-          <t>Naftali Bennett</t>
+          <t>Benny Gantz</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="0">
@@ -5814,17 +6096,17 @@
       </c>
       <c r="F8" t="inlineStr" s="0">
         <is>
-          <t>Right-wing</t>
+          <t>Centre to Centre-right</t>
         </is>
       </c>
       <c r="G8" t="inlineStr" s="0">
         <is>
-          <t>7.2</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr" s="0">
         <is>
-          <t>National conservatism, Economic liberalism, Religious-secular bridge</t>
+          <t>Statism (Mamlachtiyut), Liberal conservatism, Pragmatism</t>
         </is>
       </c>
       <c r="I8" t="inlineStr" s="0">
@@ -5836,22 +6118,22 @@
     <row r="9">
       <c r="A9" t="inlineStr" s="0">
         <is>
-          <t>YB</t>
+          <t>BENNETT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="0">
         <is>
-          <t>Yisrael Beiteinu</t>
+          <t>Bennett (B'Yachad)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="0">
         <is>
-          <t>Yisrael Beiteinu</t>
+          <t>Bennett 2026 / B'Yachad</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="0">
         <is>
-          <t>Avigdor Lieberman</t>
+          <t>Naftali Bennett</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="0">
@@ -5866,12 +6148,12 @@
       </c>
       <c r="G9" t="inlineStr" s="0">
         <is>
-          <t>7.4</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="H9" t="inlineStr" s="0">
         <is>
-          <t>Secular nationalism, Revisionist Zionism</t>
+          <t>National conservatism, Economic liberalism, Religious-secular bridge</t>
         </is>
       </c>
       <c r="I9" t="inlineStr" s="0">
@@ -5883,22 +6165,22 @@
     <row r="10">
       <c r="A10" t="inlineStr" s="0">
         <is>
-          <t>LIKUD</t>
+          <t>YB</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="0">
         <is>
-          <t>Likud</t>
+          <t>Yisrael Beiteinu</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="0">
         <is>
-          <t>Likud – National Liberal Movement</t>
+          <t>Yisrael Beiteinu</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="0">
         <is>
-          <t>Benjamin Netanyahu</t>
+          <t>Avigdor Lieberman</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="0">
@@ -5913,39 +6195,39 @@
       </c>
       <c r="G10" t="inlineStr" s="0">
         <is>
-          <t>7.6</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="H10" t="inlineStr" s="0">
         <is>
-          <t>National conservatism, Revisionist Zionism, Right-wing populism</t>
+          <t>Secular nationalism, Revisionist Zionism</t>
         </is>
       </c>
       <c r="I10" t="inlineStr" s="0">
         <is>
-          <t>Netanyahu bloc</t>
+          <t>Opposition bloc</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="0">
         <is>
-          <t>SHAS</t>
+          <t>LIKUD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="0">
         <is>
-          <t>Shas</t>
+          <t>Likud</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="0">
         <is>
-          <t>Shas (Sephardic Shomrei Torah)</t>
+          <t>Likud – National Liberal Movement</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="0">
         <is>
-          <t>Aryeh Deri</t>
+          <t>Benjamin Netanyahu</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="0">
@@ -5955,17 +6237,17 @@
       </c>
       <c r="F11" t="inlineStr" s="0">
         <is>
-          <t>Right-wing (Religiously conservative)</t>
+          <t>Right-wing</t>
         </is>
       </c>
       <c r="G11" t="inlineStr" s="0">
         <is>
-          <t>7.8</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="H11" t="inlineStr" s="0">
         <is>
-          <t>Sephardic Haredi interests, Religious conservatism, Welfare</t>
+          <t>National conservatism, Revisionist Zionism, Right-wing populism</t>
         </is>
       </c>
       <c r="I11" t="inlineStr" s="0">
@@ -5977,22 +6259,22 @@
     <row r="12">
       <c r="A12" t="inlineStr" s="0">
         <is>
-          <t>UTJ</t>
+          <t>SHAS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="0">
         <is>
-          <t>UTJ</t>
+          <t>Shas</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="0">
         <is>
-          <t>United Torah Judaism (Agudat Yisrael – Degel HaTorah)</t>
+          <t>Shas (Sephardic Shomrei Torah)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="0">
         <is>
-          <t>Yitzhak Goldknopf &amp; Moshe Gafni</t>
+          <t>Aryeh Deri</t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="0">
@@ -6007,12 +6289,12 @@
       </c>
       <c r="G12" t="inlineStr" s="0">
         <is>
-          <t>8.0</t>
+          <t>7.8</t>
         </is>
       </c>
       <c r="H12" t="inlineStr" s="0">
         <is>
-          <t>Ashkenazi Haredi interests, Halakhic conservatism</t>
+          <t>Sephardic Haredi interests, Religious conservatism, Welfare</t>
         </is>
       </c>
       <c r="I12" t="inlineStr" s="0">
@@ -6024,22 +6306,22 @@
     <row r="13">
       <c r="A13" t="inlineStr" s="0">
         <is>
-          <t>RZ</t>
+          <t>UTJ</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="0">
         <is>
-          <t>Religious Zionism</t>
+          <t>UTJ</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="0">
         <is>
-          <t>Religious Zionism (Mafdal – Tkuma)</t>
+          <t>United Torah Judaism (Agudat Yisrael – Degel HaTorah)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr" s="0">
         <is>
-          <t>Bezalel Smotrich</t>
+          <t>Yitzhak Goldknopf &amp; Moshe Gafni</t>
         </is>
       </c>
       <c r="E13" t="inlineStr" s="0">
@@ -6049,17 +6331,17 @@
       </c>
       <c r="F13" t="inlineStr" s="0">
         <is>
-          <t>Far-right</t>
+          <t>Right-wing (Religiously conservative)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr" s="0">
         <is>
-          <t>9.1</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="H13" t="inlineStr" s="0">
         <is>
-          <t>Religious Zionism, Hardline settlement expansion, Social conservatism</t>
+          <t>Ashkenazi Haredi interests, Halakhic conservatism</t>
         </is>
       </c>
       <c r="I13" t="inlineStr" s="0">
@@ -6071,45 +6353,92 @@
     <row r="14">
       <c r="A14" t="inlineStr" s="0">
         <is>
+          <t>RZ</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="0">
+        <is>
+          <t>Religious Zionism</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="0">
+        <is>
+          <t>Religious Zionism (Mafdal – Tkuma)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="0">
+        <is>
+          <t>Bezalel Smotrich</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr" s="0">
+        <is>
+          <t>2026 Knesset</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr" s="0">
+        <is>
+          <t>Far-right</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr" s="0">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr" s="0">
+        <is>
+          <t>Religious Zionism, Hardline settlement expansion, Social conservatism</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr" s="0">
+        <is>
+          <t>Netanyahu bloc</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr" s="0">
+        <is>
           <t>OY</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr" s="0">
+      <c r="B15" t="inlineStr" s="0">
         <is>
           <t>Otzma Yehudit</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr" s="0">
+      <c r="C15" t="inlineStr" s="0">
         <is>
           <t>Otzma Yehudit (Jewish Power)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr" s="0">
+      <c r="D15" t="inlineStr" s="0">
         <is>
           <t>Itamar Ben-Gvir</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr" s="0">
+      <c r="E15" t="inlineStr" s="0">
         <is>
           <t>2026 Knesset</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr" s="0">
+      <c r="F15" t="inlineStr" s="0">
         <is>
           <t>Far-right</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr" s="0">
+      <c r="G15" t="inlineStr" s="0">
         <is>
           <t>9.6</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr" s="0">
+      <c r="H15" t="inlineStr" s="0">
         <is>
           <t>Ultranationalism, Kahanism-inspired religious nationalism</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr" s="0">
+      <c r="I15" t="inlineStr" s="0">
         <is>
           <t>Netanyahu bloc</t>
         </is>

</xml_diff>